<commit_message>
upd. PCusage_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -922,10 +922,10 @@
         <v>7</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="E8" s="9">
-        <v>9397</v>
+        <v>11251</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
upd. AIusage_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="93">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t>2016-2025</t>
+  </si>
+  <si>
+    <t>2021-2025</t>
   </si>
 </sst>
 </file>
@@ -853,10 +856,10 @@
         <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>41</v>
+        <v>92</v>
       </c>
       <c r="E5" s="9">
-        <v>8605</v>
+        <v>6382</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
upd. BDusage_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -879,10 +879,10 @@
         <v>7</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>41</v>
+        <v>92</v>
       </c>
       <c r="E6" s="9">
-        <v>6456</v>
+        <v>6600</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
upd. BDusage_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -1362,10 +1362,10 @@
         <v>7</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>41</v>
+        <v>92</v>
       </c>
       <c r="E6" s="9">
-        <v>376</v>
+        <v>470</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
upd. AIusage_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="92">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -143,9 +143,6 @@
   </si>
   <si>
     <t>Число организаций, использовавших ИИ</t>
-  </si>
-  <si>
-    <t>2021-2024</t>
   </si>
   <si>
     <t>1_ОКВЭД.xlsx</t>
@@ -813,7 +810,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -824,16 +821,16 @@
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>48</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>49</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E4" s="9">
         <v>11300</v>
@@ -842,7 +839,7 @@
         <v>10</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -856,7 +853,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E5" s="9">
         <v>6382</v>
@@ -865,21 +862,21 @@
         <v>10</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E6" s="9">
         <v>6600</v>
@@ -888,21 +885,21 @@
         <v>10</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>50</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>51</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E7" s="9">
         <v>11243</v>
@@ -911,21 +908,21 @@
         <v>10</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E8" s="9">
         <v>11251</v>
@@ -934,7 +931,7 @@
         <v>10</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -962,7 +959,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -1019,7 +1016,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1039,7 +1036,7 @@
         <v>23</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E14" s="4">
         <v>4084</v>
@@ -1062,7 +1059,7 @@
         <v>23</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E15" s="4">
         <v>9211</v>
@@ -1085,7 +1082,7 @@
         <v>23</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E16" s="4">
         <v>1915</v>
@@ -1108,7 +1105,7 @@
         <v>23</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E17" s="4">
         <v>4260</v>
@@ -1191,7 +1188,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -1202,16 +1199,16 @@
     </row>
     <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="21" t="s">
         <v>55</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>56</v>
       </c>
       <c r="C22" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E22" s="20">
         <v>1207</v>
@@ -1220,15 +1217,15 @@
         <v>10</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>58</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>59</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>23</v>
@@ -1243,7 +1240,7 @@
         <v>10</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1268,7 +1265,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1296,7 +1293,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -1307,10 +1304,10 @@
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>7</v>
@@ -1322,15 +1319,15 @@
         <v>752</v>
       </c>
       <c r="F4" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>62</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>40</v>
@@ -1339,47 +1336,47 @@
         <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>41</v>
+        <v>91</v>
       </c>
       <c r="E5" s="9">
-        <v>376</v>
+        <v>470</v>
       </c>
       <c r="F5" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>62</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E6" s="9">
         <v>470</v>
       </c>
       <c r="F6" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>62</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -1391,18 +1388,18 @@
         <v>752</v>
       </c>
       <c r="F7" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>62</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
@@ -1414,15 +1411,15 @@
         <v>752</v>
       </c>
       <c r="F8" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>62</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>5</v>
@@ -1437,15 +1434,15 @@
         <v>658</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -1456,7 +1453,7 @@
     </row>
     <row r="11" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>11</v>
@@ -1471,15 +1468,15 @@
         <v>658</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>15</v>
@@ -1494,15 +1491,15 @@
         <v>846</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1513,7 +1510,7 @@
     </row>
     <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>22</v>
@@ -1522,21 +1519,21 @@
         <v>23</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E14" s="4">
         <v>188</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>26</v>
@@ -1545,21 +1542,21 @@
         <v>23</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E15" s="4">
         <v>940</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>28</v>
@@ -1568,21 +1565,21 @@
         <v>23</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E16" s="4">
         <v>526</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>31</v>
@@ -1591,21 +1588,21 @@
         <v>23</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E17" s="4">
         <v>939</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>33</v>
@@ -1620,15 +1617,15 @@
         <v>846</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>37</v>
@@ -1643,15 +1640,15 @@
         <v>846</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>38</v>
@@ -1666,15 +1663,15 @@
         <v>846</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -1685,10 +1682,10 @@
     </row>
     <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C22" s="20" t="s">
         <v>23</v>
@@ -1700,18 +1697,18 @@
         <v>752</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>75</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>76</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>23</v>
@@ -1723,10 +1720,10 @@
         <v>846</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
upd. ITusage_r, PCusage_r and inetusage_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -1313,10 +1313,10 @@
         <v>7</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E4" s="9">
-        <v>752</v>
+        <v>846</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>61</v>
@@ -1382,10 +1382,10 @@
         <v>7</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E7" s="9">
-        <v>752</v>
+        <v>846</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>61</v>
@@ -1405,10 +1405,10 @@
         <v>7</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E8" s="9">
-        <v>752</v>
+        <v>846</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
upd. RDcosts_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -1128,10 +1128,10 @@
         <v>23</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="E18" s="4">
-        <v>1660</v>
+        <v>1297</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
upd. RDsalary_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -1151,10 +1151,10 @@
         <v>23</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="E19" s="4">
-        <v>1658</v>
+        <v>1287</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
upd. RDequip_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -1174,10 +1174,10 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="E20" s="4">
-        <v>1656</v>
+        <v>753</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
upd. RDcosts_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -1611,10 +1611,10 @@
         <v>23</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E18" s="4">
-        <v>846</v>
+        <v>922</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
upd. RDsalary_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -1634,10 +1634,10 @@
         <v>23</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E19" s="4">
-        <v>846</v>
+        <v>922</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
upd. RDequip_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -1657,10 +1657,10 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E20" s="4">
-        <v>846</v>
+        <v>829</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
upd. researchersavg_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="93">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t>2021-2025</t>
+  </si>
+  <si>
+    <t>2018-2025</t>
   </si>
 </sst>
 </file>
@@ -979,10 +982,10 @@
         <v>13</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>8</v>
+        <v>92</v>
       </c>
       <c r="E11" s="14">
-        <v>1567</v>
+        <v>1345</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
upd. researchorg_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -948,10 +948,10 @@
         <v>7</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>8</v>
+        <v>92</v>
       </c>
       <c r="E9" s="16">
-        <v>1567</v>
+        <v>2135</v>
       </c>
       <c r="F9" s="16" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
upd. researchorg_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -1431,10 +1431,10 @@
         <v>7</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>8</v>
+        <v>92</v>
       </c>
       <c r="E9" s="16">
-        <v>658</v>
+        <v>752</v>
       </c>
       <c r="F9" s="24" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
upd. researchersavg_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="92">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -44,9 +44,6 @@
   </si>
   <si>
     <t>ед.</t>
-  </si>
-  <si>
-    <t>2018-2024</t>
   </si>
   <si>
     <t xml:space="preserve">Структура </t>
@@ -785,7 +782,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -805,15 +802,15 @@
         <v>3</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -824,117 +821,117 @@
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>47</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>48</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E4" s="9">
         <v>11300</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>39</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>40</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E5" s="9">
         <v>6382</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>42</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>43</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E6" s="9">
         <v>6600</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>49</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>50</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E7" s="9">
         <v>11243</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>51</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>52</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E8" s="9">
         <v>11251</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -948,21 +945,21 @@
         <v>7</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E9" s="16">
         <v>2135</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -973,53 +970,53 @@
     </row>
     <row r="11" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>13</v>
-      </c>
       <c r="D11" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E11" s="14">
         <v>1345</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="14" t="s">
         <v>16</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>17</v>
       </c>
       <c r="E12" s="14">
         <v>1707</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1030,168 +1027,168 @@
     </row>
     <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>23</v>
-      </c>
       <c r="D14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E14" s="4">
         <v>4084</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="C15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E15" s="4">
         <v>9211</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E16" s="4">
         <v>1915</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E17" s="4">
         <v>4260</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E18" s="4">
         <v>1297</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E19" s="4">
         <v>1287</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E20" s="4">
         <v>753</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -1202,48 +1199,48 @@
     </row>
     <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="C22" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="20" t="s">
         <v>55</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>56</v>
       </c>
       <c r="E22" s="20">
         <v>1207</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>58</v>
-      </c>
       <c r="C23" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E23" s="20">
         <v>513</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1268,7 +1265,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1288,15 +1285,15 @@
         <v>3</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -1307,122 +1304,122 @@
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E4" s="9">
         <v>846</v>
       </c>
       <c r="F4" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E5" s="9">
         <v>470</v>
       </c>
       <c r="F5" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E6" s="9">
         <v>470</v>
       </c>
       <c r="F6" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E7" s="9">
         <v>846</v>
       </c>
       <c r="F7" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E8" s="9">
         <v>846</v>
       </c>
       <c r="F8" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>5</v>
@@ -1431,21 +1428,21 @@
         <v>7</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E9" s="16">
         <v>752</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -1456,53 +1453,53 @@
     </row>
     <row r="11" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>8</v>
+        <v>91</v>
       </c>
       <c r="E11" s="14">
-        <v>658</v>
+        <v>742</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E12" s="14">
         <v>846</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1513,168 +1510,168 @@
     </row>
     <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>23</v>
-      </c>
       <c r="D14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E14" s="4">
         <v>188</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E15" s="4">
         <v>940</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E16" s="4">
         <v>526</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E17" s="4">
         <v>939</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E18" s="4">
         <v>922</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E19" s="4">
         <v>922</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E20" s="4">
         <v>829</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -1685,48 +1682,48 @@
     </row>
     <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E22" s="20">
         <v>752</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>75</v>
-      </c>
       <c r="C23" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E23" s="20">
         <v>846</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
upd. researchers_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -1002,10 +1002,10 @@
         <v>12</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="E12" s="14">
-        <v>1707</v>
+        <v>1391</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
upd. researchers_r (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -1485,10 +1485,10 @@
         <v>12</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>26</v>
+        <v>89</v>
       </c>
       <c r="E12" s="14">
-        <v>846</v>
+        <v>924</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
upd. VDS_s (data for 2025)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -1231,10 +1231,10 @@
         <v>22</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>26</v>
+        <v>89</v>
       </c>
       <c r="E23" s="20">
-        <v>513</v>
+        <v>570</v>
       </c>
       <c r="F23" s="20" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
upd. factoriescap_r (data for 2025 and corr)
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="91">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -70,9 +70,6 @@
     <t>researchers_s</t>
   </si>
   <si>
-    <t>2017-2024</t>
-  </si>
-  <si>
     <t>11_ОКВЭД2_публ.xlsx</t>
   </si>
   <si>
@@ -247,33 +244,6 @@
     <t>Валовая добавленная стоимость по регионам РФ</t>
   </si>
   <si>
-    <r>
-      <t>Объем отгруженных товаров собственного производства, выполненных работ и услуг собственными силами (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>СУММА</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
     <t>factoriescap_r</t>
   </si>
   <si>
@@ -320,6 +290,9 @@
   </si>
   <si>
     <t>2018-2025</t>
+  </si>
+  <si>
+    <t>Объем отгруженных товаров собственного производства, выполненных работ и услуг собственными силами</t>
   </si>
 </sst>
 </file>
@@ -805,12 +778,12 @@
         <v>8</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -821,16 +794,16 @@
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>46</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>47</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E4" s="9">
         <v>11300</v>
@@ -839,21 +812,21 @@
         <v>9</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>38</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>39</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E5" s="9">
         <v>6382</v>
@@ -862,21 +835,21 @@
         <v>9</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>41</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>42</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E6" s="9">
         <v>6600</v>
@@ -885,21 +858,21 @@
         <v>9</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>48</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>49</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E7" s="9">
         <v>11243</v>
@@ -908,21 +881,21 @@
         <v>9</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>50</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>51</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E8" s="9">
         <v>11251</v>
@@ -931,7 +904,7 @@
         <v>9</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -945,7 +918,7 @@
         <v>7</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E9" s="16">
         <v>2135</v>
@@ -954,12 +927,12 @@
         <v>9</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -979,7 +952,7 @@
         <v>12</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E11" s="14">
         <v>1345</v>
@@ -988,7 +961,7 @@
         <v>9</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -1002,7 +975,7 @@
         <v>12</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E12" s="14">
         <v>1391</v>
@@ -1011,12 +984,12 @@
         <v>9</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1027,16 +1000,16 @@
     </row>
     <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="D14" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E14" s="4">
         <v>4084</v>
@@ -1045,21 +1018,21 @@
         <v>9</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>25</v>
-      </c>
       <c r="C15" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E15" s="4">
         <v>9211</v>
@@ -1068,21 +1041,21 @@
         <v>9</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E16" s="4">
         <v>1915</v>
@@ -1091,21 +1064,21 @@
         <v>9</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E17" s="4">
         <v>4260</v>
@@ -1114,21 +1087,21 @@
         <v>9</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E18" s="4">
         <v>1297</v>
@@ -1137,21 +1110,21 @@
         <v>9</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E19" s="4">
         <v>1287</v>
@@ -1160,21 +1133,21 @@
         <v>9</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E20" s="4">
         <v>753</v>
@@ -1183,12 +1156,12 @@
         <v>9</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -1199,16 +1172,16 @@
     </row>
     <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="C22" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" s="20" t="s">
         <v>54</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>55</v>
       </c>
       <c r="E22" s="20">
         <v>1207</v>
@@ -1217,21 +1190,21 @@
         <v>9</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>57</v>
-      </c>
       <c r="C23" s="20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E23" s="20">
         <v>570</v>
@@ -1240,7 +1213,7 @@
         <v>9</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1265,7 +1238,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1288,12 +1261,12 @@
         <v>8</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -1304,122 +1277,122 @@
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E4" s="9">
         <v>846</v>
       </c>
       <c r="F4" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E5" s="9">
         <v>470</v>
       </c>
       <c r="F5" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E6" s="9">
         <v>470</v>
       </c>
       <c r="F6" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E7" s="9">
         <v>846</v>
       </c>
       <c r="F7" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E8" s="9">
         <v>846</v>
       </c>
       <c r="F8" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>5</v>
@@ -1428,21 +1401,21 @@
         <v>7</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E9" s="16">
         <v>752</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -1453,7 +1426,7 @@
     </row>
     <row r="11" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>10</v>
@@ -1462,21 +1435,21 @@
         <v>12</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E11" s="14">
         <v>742</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>14</v>
@@ -1485,21 +1458,21 @@
         <v>12</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E12" s="14">
         <v>924</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1510,168 +1483,168 @@
     </row>
     <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="D14" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E14" s="4">
         <v>188</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E15" s="4">
         <v>940</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E16" s="4">
         <v>526</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E17" s="4">
         <v>939</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E18" s="4">
         <v>922</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E19" s="4">
         <v>922</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E20" s="4">
         <v>829</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -1682,48 +1655,48 @@
     </row>
     <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E22" s="20">
-        <v>752</v>
+        <v>846</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>74</v>
-      </c>
       <c r="C23" s="20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E23" s="20">
         <v>846</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update description of features.xlsx
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
-    <sheet name="По регионам" sheetId="2" r:id="rId2"/>
+    <sheet name="По отраслям RU" sheetId="1" r:id="rId1"/>
+    <sheet name="По регионам RU" sheetId="2" r:id="rId2"/>
+    <sheet name="По регионам KZ" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="99">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -293,6 +294,30 @@
   </si>
   <si>
     <t>Объем отгруженных товаров собственного производства, выполненных работ и услуг собственными силами</t>
+  </si>
+  <si>
+    <t>VDS_r.kz</t>
+  </si>
+  <si>
+    <t>Признаки по регионам Казахстана (приставка _r - region, .kz - Казахстан)</t>
+  </si>
+  <si>
+    <t>Валовая добавленная стоимость малого и среднего предпринимательства по регионам</t>
+  </si>
+  <si>
+    <t>млн. тенге</t>
+  </si>
+  <si>
+    <t>2005-2024</t>
+  </si>
+  <si>
+    <t>region, year, value</t>
+  </si>
+  <si>
+    <t>Исходник-форма</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Бюро национальной статистики (отраслевая статистика, статистика предприятий) </t>
   </si>
 </sst>
 </file>
@@ -372,7 +397,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -395,11 +420,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -460,6 +511,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1703,4 +1763,88 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.7109375" customWidth="1"/>
+    <col min="2" max="2" width="47.5703125" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" customWidth="1"/>
+    <col min="7" max="7" width="38.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+    </row>
+    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" s="20">
+        <v>356</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>98</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update description of features
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="106">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -327,6 +327,18 @@
   </si>
   <si>
     <t xml:space="preserve">Бюро национальной статистики (Об инновационной деятельности предприятий в Республике Казахстан) </t>
+  </si>
+  <si>
+    <t>inetusage_r.kz</t>
+  </si>
+  <si>
+    <t>Количество организаций, использующих сеть Интернет</t>
+  </si>
+  <si>
+    <t>2004-2025</t>
+  </si>
+  <si>
+    <t>Бюро национальной статистики (информационно-коммуникационные технологии)</t>
   </si>
 </sst>
 </file>
@@ -459,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -524,13 +536,16 @@
     <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1779,7 +1794,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.7109375" customWidth="1"/>
@@ -1820,8 +1835,8 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="26"/>
-      <c r="B3" s="27"/>
+      <c r="A3" s="27"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="19"/>
       <c r="D3" s="19"/>
       <c r="E3" s="19"/>
@@ -1855,7 +1870,7 @@
       <c r="A5" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="26" t="s">
         <v>100</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -1872,6 +1887,29 @@
       </c>
       <c r="G5" s="6" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="E6" s="29">
+        <v>406</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="G6" s="29" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>